<commit_message>
Implementar selección de categoría en el scraper: se añade la función `select_category` para permitir al usuario elegir o crear categorías. Se actualiza la clase `ExcelHandler` para manejar múltiples hojas por categoría y se mejora la gestión de productos en Excel.
</commit_message>
<xml_diff>
--- a/productos_mercadolibre.xlsx
+++ b/productos_mercadolibre.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="almacenamiento" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monitores" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,71 +430,276 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>precio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>precio_anterior</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>descuento</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>envio</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>envio_gratis</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>total_reviews</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>imagen</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_actualizacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ssd Nvme Disco Duro Solido 512 Gb M2 2280 Laptop Computacion</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=ee0j4wvh3eoimsVzRTuAIAVGZRhEh39tccNpGmJsQsTUTvaZtOkuMFEVDCpA1wo7L9E1Qcv4mZQjQW4t0%2BpzVZGZ02sRp9HovJI4gnDsJ57b2KbH2A97ga%2FuHfWF98KKSMI78U9iYOyiJc45zf26KS%2B7VFk0dbFL4PrNuBCoaKkLh%2FWuYqqohEj70HEkOey5n%2FlaNCLBf%2BRjNL9HCjnYIDnfJTp5SLOsupH6LYnRR5PObE2tTdhe%2BPLZyj4JNYaDPjhaw%2BfcxUA%2FjA0yyCdr%2Be5yiFe8ljZcO356%2Bx5%2FQuvehjUTrO2lYmJyL0y4jwwVa79L7wbm%2FOx9BkmPoIiscJx5IwCMBXfsDNxiphyxc02mDpvf1SenSh0CeCeOE4GDQvb6cW8hx9WKKgHtI6lNQ%2F7bYaQlym%2FANBX%2FJAuRJFe1appHjiOU3N8xz2jGJh5ZSokVbB0rnJOy1d7JPFZAxZ4Ub50%2FHR%2FIAXNxW7ZV7oOnBDrK4vRK8WOQfDCMSJGuBqIdQsplAbZToNITHwKtS9VrPvfiMMEAqbwYrqNjNR%2FgL5dhCy1BTCiXGh4%2FkThcWUcoCQqOtOUm2m1Rp2%2B7COiH4u5D3CmY%2BUEU8iwY9RmHq4zdxGXnifZE9qQohxhpMf0fXo1qFAz1NblBF%2BdWDmRw2A68Bi%2F%2B8mCUqG1XYyuCO9Mjmkxrrz9pnxGEXB10EfDRNjbF7jjGGRNecoDH%2BT5R4nWK2XgCDCo9gX1qyoDgt%2Bgbor0Yy1rHD9GCCmTfZIZvNyOCKaJkxtEz2RxWUwrkO1bQN7vpO%2F5Hbg%3D%3D&amp;highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=eb85adee-7abb-4fdd-ab55-264cf6b14e7e&amp;wid=MCO2742971682&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>176560</v>
+      </c>
+      <c r="E2" t="n">
+        <v>296500</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>40% OFF</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J2" t="n">
+        <v>14</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_764117-MCO83036481287_032025-V.webp</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>45809.63719189815</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Disco Solido Ssd Interno 120gb (128gb) Sata Premium Seguro</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=t80usphhHp4v1mI6O87K82wGWIJ3bYXyjr3NaWgzhLEiq75tvWqauIq6Ycr%2BVjLTRyjU4H9F%2BqKKM3EOLQC2mhzWa1e6tlTDXqzGXLEOCpzxC6gwqvTrjHKkVyigls4VW9hvoUR%2FnVM7Tjvp0obKB3o61fK4EIgx0IdJKVuPpU0fhXocfiy6C6uXXpAqHM8OBUwBurVGvO7K%2FY5dNrQZ4%2FTVKslVDBx%2F7LlLcIXc9LwbXjdXpzPml6rNxP1ksjouCirVNSscccUrNItopUGPTk931pNnoDISw%2Bda2CKVt8YgawivOKx6h0XiBWHPRNVVJbCQegnEVUPSpCHiZFnTTUphrV4MLuCWzMHy%2FVePCofQrwxecBzSrCg2v%2FyF7AX%2FaHgSI%2BSiuQu5T5hYNMjIW9dhivsDPb7BlJa8W4Wq5wdNnX1lWFyLFBhnCw2f0jf95PQXir%2FYhgosOok5NP2GluGvq78WuvpbWY6S%2Bhve871eb6O0lUoQpg5jXDGsPKC7yh0ujo56VTtH78uctTGWUWpG41vTNHyQD05%2BbqIDIMubBomVr5qTTDINoyVER61zjA517kFRFJ7drd0qRkjcMKGPRuUL2BVwxftBiIQ40jC8ez5IxXVuhhZqlpcfkij4guH5JJHl3Cc5pywwSsera%2BQdu60a%2Bw0IsIjbofcBYUUAg7YhVGCfkbI6AZa6rgmYPrPm2VgkNF%2FbntVRLXON%2FnMW%2B3tfIfoyDxxbJVp1P0X8iisw%2FQSN9Xar%2B0r%2F9rarpmSBL5BODeHAPWh3LxULfoer21jY4K%2BjXvAWe%2FemSmDMDZFtVENWgGWvRu5AO9PqC4LmyTI9N%2F83v7QMD%2F5NPbJyMNtXzXbNiCoruxRtco%2FORiFCpIFOSg%3D%3D&amp;searchVariation=173636587098&amp;highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=eb85adee-7abb-4fdd-ab55-264cf6b14e7e</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>49600</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_667991-MCO54907943874_042023-V.webp</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>45809.63719193287</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADATA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Disco sólido SSD interno Adata Ultimate SU650 ASU650SS-512GT-R 512GB</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/disco-solido-ssd-interno-adata-ultimate-su650-asu650ss-512gt-r-512gb/p/MCO35339869?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO35339869&amp;position=6&amp;search_layout=stack&amp;type=product&amp;tracking_id=eb85adee-7abb-4fdd-ab55-264cf6b14e7e&amp;wid=MCO2329119764&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>142900</v>
+      </c>
+      <c r="E4" t="n">
+        <v>299888</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>52% OFF</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>696</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>45809.63719194444</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>marca</t>
         </is>
       </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>titulo</t>
+          <t>url</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>url</t>
+          <t>precio</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>precio</t>
+          <t>precio_anterior</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>precio_anterior</t>
+          <t>descuento</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>descuento</t>
+          <t>envio</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>envio</t>
+          <t>envio_gratis</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>envio_gratis</t>
+          <t>rating</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>rating</t>
+          <t>total_reviews</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>total_reviews</t>
+          <t>imagen</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>imagen</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>fecha_actualizacion</t>
         </is>
@@ -502,178 +708,217 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lapto</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>Monitor Gamer Xiaomi con pantalla de 34" 180Hz 110V y resolución WQHD</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Computador Portatil Laptop Corporativo Promocion Usado</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=%2FteWDOW%2FleiSB2FF9%2BdNlL4T4Qo3T6DDutkHIgD8Yx5xBxfC6QplCKVQ1uVGOtTxpEajBXGloX%2FE7SCQyJhGo9xnIIr72dhXoDek%2BHHuzoUothCKDXBsEudoaU0ulpCiYRvQI%2BHTIWSNE%2BhWzczLyhoTTgYKespsg3q3jKHk33Syf0NQBwXwZL%2FP1wHhsO0YKPArxia1j4OOvZx0oZzLxid12cmF3fQHArtEp1m7jhJiZBr%2BdqRem9mVIikk6%2FNC6kwqgbRLAgh7oC4GqwG1i3N%2Fer9%2BoXZeojjx04edyZpWCJ2Gk60AwgyKHHZSjSLybaTDfJfcDoKxjWtOZ9WN2EjWzr9gD775Mzdc77PUM%2FC2sB9jJmg0oewUJa3xG18fjFDVrbaoqzB0Rm30X8URPQG%2FibvFXmkMSvfWWP2vmkkbHGaUU0Pf2eiLm1aQmkoACgjIOphPBs%2BxQRgMnAf3kcpQlJ2eClc43wK3gifuJ9ZdaYXpOcUUbjQtIsLlwFqyAilUc8OjNSCIp%2Bh5R%2B%2FE5EKV32fSlxYvTB13iZIYVMtjGTDK3W3goMX90m6qdVJPicqXNVEt9EpmknGrceichQJ6GBjDQ3O4PwpeMx%2ByPFilhfl8YmFeaLGXXNKJcezUM%2BusVA%2FJGWf85RWkAy5kmUs4F6q3hl%2F0kF4%2Be2bjKF1w430S9LHlp6UIUxHYlatnuwUCf%2B9KtRWo%2FaJ4g%2B7PA3dHP%2BVCBTFtv9RoyCcmKF0pz2AaEnowFcZlE9eobkLm2qkHIlDIAml1FXUj6ZARYOlnMFeGgqml4aIPEaGAFdJoToKPixCg078dTX2Xkahw28Vb94xQHotV8b9Qkx8zMTiL8Xmx8ApWjntW7bvvrNSncAPOt%2FKCGg%3D%3D&amp;searchVariation=181673730321&amp;highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=6d1f0b94-94af-437e-9b51-a8647a004bfd</t>
-        </is>
+          <t>https://www.mercadolibre.com.co/monitor-gamer-xiaomi-con-pantalla-de-34-180hz-110v-y-resolucion-wqhd/p/MCO43960788?highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO43960788&amp;position=4&amp;search_layout=stack&amp;type=product&amp;tracking_id=1615f080-5283-4342-a0d2-599a57689da2&amp;wid=MCO1518847209&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1513122</v>
       </c>
       <c r="E2" t="n">
-        <v>759999</v>
-      </c>
-      <c r="F2" t="n">
-        <v>999999</v>
+        <v>1949900</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>22% OFF</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>24% OFF</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>Envío gratis</t>
         </is>
       </c>
-      <c r="I2" t="b">
+      <c r="H2" t="b">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>58</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://http2.mlstatic.com/D_Q_NP_2X_762946-MCO83338686127_032025-V.webp</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>45809.63341739828</v>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_827699-MLU74975109969_032024-V.webp</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>45809.63902657673</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lapto</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Monitor LG curvo 32MR50C-B Full HD 32" 1920 px x 1080 px negro 110V</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Laptop Hp I5 Ddr4 8gb Ssd 240gb Windows 11</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=rBE1tT%2BhBOdV1aiCUdqCp%2BJ284SSmHG65dYuVQ4Gm58xYdoBb8Ygv9dfBMflJv%2BJr%2Bnz55gMvHnWgK%2B1k3NX90A6uE%2BVjZDezWjthR1Wmkt0aymXZdivKLT%2BewhVsX6Gnn5T5d%2FScxLjInMP1nCf9QKpW%2FhrW5vdjpl7tsE%2B5F6fqbcxqZ7ZVc%2FNowh4QbQzOjfcEIOor9p16mbTL6iS3VJkTXPpi8rOT0MSXJxTlR1w12n4rYAjlM9KiUZROn%2Bq7ramlmGtNQNJHBOLTCTr9CjWSocjPD0S4xbt5tr9248dbxiQScquMa3hkSXWst9WTZ6gOyVXBJR9G%2FE68V1knb9zHyVOq5mk%2FWDks2S5pKFOB9TKUHNXlnMkDm%2Bwq2aTW9MVM%2B2crskT0AqAHINtL82s1Bb7zZBlSLPeOa98m8yNxK0pxOSvkG4EWdCHf%2BePXGjh12q9%2BYdVKxtFm4OEZb9AT1L2lctqTqlMKlXrDJxn5H8DYSexheaJGV%2FKjNGVTX0SKFdyl7x1C%2Fxcra6mUNu4BnWhqeHl85gTonlD25cNIvpUzLMjSaPoWtRaFfQ9WKn366zrxVBb1B7g0meUC7YsIU9Mo2g8gHBJKes%2BbCWeeWdzL1rzv9qdUvTQeIOKUY%2FSbp2XMMsUD4AP67fX6bvsHtlA%2Bf0MGvuH8QFFvw60TIf4iVQTM%2FNcrqsLkAY5gnhyFaJe8Mc5cKRvEInQkxxRtLXhNFtn1GwAFQ4WqEQ8RgTvgc9stfK0ccFZEHU%2B%2F%2BOSw1n9ZqO%2FCY%2FfaMR0qomvBIv7rTOxVc7emMZ%2BbGPbCPz7nQ5klJD3lr48VLk4F6Zia6Dg%2FWgcdbIRwkw1n0O1YNAdqijZsfM%3D&amp;searchVariation=186865852637&amp;highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=6d1f0b94-94af-437e-9b51-a8647a004bfd</t>
-        </is>
+          <t>https://www.mercadolibre.com.co/monitor-lg-curvo-32mr50c-b-full-hd-32-1920-px-x-1080-px-negro-110v/p/MCO38243621?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO38243621&amp;position=5&amp;search_layout=stack&amp;type=product&amp;tracking_id=1615f080-5283-4342-a0d2-599a57689da2&amp;wid=MCO1578787515&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>780000</v>
       </c>
       <c r="E3" t="n">
-        <v>769999</v>
-      </c>
-      <c r="F3" t="n">
-        <v>999999</v>
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>23% OFF</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>Envío gratis</t>
         </is>
       </c>
-      <c r="I3" t="b">
+      <c r="H3" t="b">
         <v>1</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>65</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>https://http2.mlstatic.com/D_Q_NP_2X_966418-MCO84722083030_052025-V.webp</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>45809.63341744232</v>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_663594-MLU77449045398_072024-V.webp</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>45809.63902660412</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>lapto</t>
+          <t>SAMSUNG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASUS</t>
+          <t>Monitor Gamer Samsung C27R500FHL con pantalla de 27" 60Hz 110V y resolución Full HD Negro</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Portátil Asus Vivobook X1502 Ci5-12500h 24gb Ssd512 Fhd15.6 color Quiet Blue</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.mercadolibre.com.co/portatil-asus-vivobook-x1502-ci5-12500h-24gb-ssd512-fhd156-color-quiet-blue/p/MCO47191661?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO47191661&amp;position=10&amp;search_layout=stack&amp;type=product&amp;tracking_id=6d1f0b94-94af-437e-9b51-a8647a004bfd&amp;wid=MCO1569451947&amp;sid=search</t>
-        </is>
+          <t>https://www.mercadolibre.com.co/monitor-gamer-samsung-c27r500fhl-con-pantalla-de-27-60hz-110v-y-resolucion-full-hd-negro/p/MCO43958520?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO43958520&amp;position=6&amp;search_layout=stack&amp;type=product&amp;tracking_id=1615f080-5283-4342-a0d2-599a57689da2&amp;wid=MCO2766968630&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>636800</v>
       </c>
       <c r="E4" t="n">
-        <v>1929900</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2249000</v>
+        <v>1000000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>36% OFF</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>14% OFF</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>Envío gratis</t>
         </is>
       </c>
-      <c r="I4" t="b">
+      <c r="H4" t="b">
         <v>1</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>616</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
           <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>45809.63341746163</v>
+      <c r="L4" s="2" t="n">
+        <v>45809.63902661313</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Monitor gamer curvo Samsung LED dark blue gray 110V C32R500</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/monitor-gamer-curvo-samsung-led-dark-blue-gray-110v-c32r500/p/MCO43959782?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO43959782&amp;position=7&amp;search_layout=stack&amp;type=product&amp;tracking_id=1615f080-5283-4342-a0d2-599a57689da2&amp;wid=MCO2223865356&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>792900</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>343</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>45809.63902662089</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar filtros de envío en el scraper: se implementa la función `get_shipping_filters` para permitir al usuario seleccionar filtros de envío. Se actualiza la función `scrape_mercadolibre` para incluir estos filtros en la búsqueda y se modifica la clase `ExcelHandler` para registrar productos con envío Full y gratis.
</commit_message>
<xml_diff>
--- a/productos_mercadolibre.xlsx
+++ b/productos_mercadolibre.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="almacenamiento" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monitores" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="laptos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -706,11 +707,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Monitor Gamer Xiaomi con pantalla de 34" 180Hz 110V y resolución WQHD</t>
@@ -740,15 +737,11 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>4.9</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
+      <c r="I2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J2" t="n">
+        <v>58</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -756,7 +749,7 @@
         </is>
       </c>
       <c r="L2" s="2" t="n">
-        <v>45809.63902657673</v>
+        <v>45809.63902657408</v>
       </c>
     </row>
     <row r="3">
@@ -781,11 +774,7 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Envío gratis</t>
@@ -794,15 +783,11 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>4.6</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
+      <c r="I3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>65</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -810,7 +795,7 @@
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>45809.63902660412</v>
+        <v>45809.6390266088</v>
       </c>
     </row>
     <row r="4">
@@ -848,15 +833,11 @@
       <c r="H4" t="b">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>4.9</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>616</t>
-        </is>
+      <c r="I4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>616</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -864,7 +845,7 @@
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>45809.63902661313</v>
+        <v>45809.6390266088</v>
       </c>
     </row>
     <row r="5">
@@ -889,36 +870,1249 @@
       <c r="E5" t="n">
         <v>0</v>
       </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J5" t="n">
+        <v>343</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>45809.63902662037</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>precio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>precio_anterior</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>descuento</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>envio</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>envio_gratis</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>envio_full</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>total_reviews</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>imagen</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_actualizacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Portatil Hp 12ava Gen Intel I3 1215u Ssd 512gb Ram 8gb Color Plateado</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=zQFU5BvnvqwRvMq1By5NRGFlzAqpbowk3qmAcnB%2BMJNDDwXDw3blW2x0QBWMcSaSHbHCVFn8z9QnYq1eJ4%2BiIrQdn2pihRo7erq%2FCWpkfyfGrhZe5Q0y9aSLBaAyFrwBVz8pHLUl0v%2BDgI5Z4uNAxCi%2Ftq9munKuJSr3tHuxxID%2FLfS5lpjCKXZf6y5BWLNFa3o8Q9HLMLnEtrWH6sCfv8n9sIlSn%2FxupheY5iO9EiTiB82RqwRYzDEaqFAhTHmbnJTLGJES%2FduL%2BytUQ2CcXDdQ%2FI9qzFtDZuET4I7n7jCACxvJlD0TjaRS%2Bz6FWkNFiVwXpekgIj0EOvfRaJdcptKXGmGbQTHwEt3aIKw8zUwgNEXsM4WAVIvJkEg%2BAOJPiGLcvy9oLbvDE3%2F1Qg1k6L1b07xhQBYOrqJ1Hzw24XIyxvPLHuATlo1tgOMKwmDZj9pNqAuGPVH%2BsxXE8vxGcztIWVIcp8XGXGyr9hpFvVbzfH42HleBpg13sXKRJ5Vjl9lbffaiO5XWuezBmpuJUyoO4DU1nnYNjxCiyUkBOZMsxLHvpEC6G6ifDchjVYhzBo%2BzI2b1%2Fy2r5u9GyQkXGIGRacKYr9hSvlpvLDLPPndYK0kmPApJzRiDE2I1bGnupjy7MbI82xT1KZtDG29siTpEsfBaMpDYtyW2rWqdVzlvBXAmLLiFE%2BRuudIIjRhhVSuQiZjL%2FJMBEUxwP%2FSECQDekZ3LKjkiSN5%2BCqQIABFqmw%2B2FC%2FQwLH5PIoV9jos7xgpGEhBkPSPLSGW8%2Bqjfb5J7hxgYnUIh%2BYWauaZa3Gr9qgWtHoQBjKxT5y5T2Fdbu3oJnCinh1GRNPJn6XClwRyw%2FWXJCAC0F8cbL7vlQWFkgYHjQeiwyUKEVqENuIutnP7QegOWK2gdDux1vQDdxDBQ22FK56BT%2Felqvcnx%2FTeewGBs%2BJX2kTVDc4H4%2BXJehllU62pKGU4tXUI&amp;highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1507088307&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1458900</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1853000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>21% OFF</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_645989-MLU78944581522_092024-V.webp</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>45809.67502480594</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Notebook Hp 245 G10 R3 7330u 512gb Ssd 8gb Ram Windows 11 Ho</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=P218uynAcTyZmXvon7VW%2BB05NKdbrv2OpL%2FWCxMohF7wPq3pLnEW0GZVqp3NYJ8aqjTMwyMLpfrySzH1v1mRqq6ngqRFHwLD0GDtrD2hSY0Bbq4UZyhV5HSo0i0hX5StFbtvN3LkYOzknOfOMKR8UqMLlNQOoPnvDbE2hsAOTKxYOopK16M9GSZyqp%2FsqCsoexPDq1v3uFyJ2R%2BxHd7bDF%2B%2Fpr2AsZ1aWmUPSw9PmEmdYPzNpvI7e%2FKHVU88pGOs7ril5A2GpEWjzxfdOyqyDWHBjGnHtDHvxZ4UaAlJMaSRpfpUYx0Ys82tyPbnXrrYKowZIIAPGoQiAycX8FMp44x9dJgSxXznOWEL4H1h67ZcwXXtzT5jMyZyVLu5k2rEPbuH795zcKSJnK4qoKYW%2FMtvKs12XgUk0EcC1hjkLRcQ5DcSBTU1wIb1k4aq%2FvbASZYA0%2FU%2FX8LP9fEymdEy9ISan3aB3RD77qskxltzsRMqsxJZOZJ%2B3Ko%2B2W4%2F5DtESs%2FQ1%2Fzm8U4heIk2shJc0s3nRyfwJ7Jp83xnyzlMma7aQFDXhlkDT%2BKTxbWBhOt4nGugEC7PSIHNHtd7jsFocxCzKApEpr93h407loa%2B8FVCzEa%2FSGThzAlC2o6pXSgnbpjmyzBmTyW%2B4Qi9rjbGy94HiUCAJLvvEhh5vMCorTDzHBCJviWXBA0LRp8%2FPHSI8xmQzej%2FW7SLsfuvWeh8j9kMa22oCGt%2FUXpGqymoygpcwDuu2IuUcrxU6uFudy7ubRWqOjw1AYSldcCzfxhEjro2A5SJ5UzP2OvHf4EIB79MguWxk8XDyALruJtEIxE690lkCyLzU6ljjZuAAKD41fnfiGNEygW9uLZJ4Ja41lIEiWKEGc9pSg%2BkH9fM5ZE5Ggo2GeqBKnVNAyY4UDhKPJQZkioHfx6yFWBdDR1r6ayVSDeQW7wIDQtYrJ1CPmXIzA%3D%3D&amp;highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1547113843&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1259900</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1621375</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>22% OFF</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_679019-MLU78080956988_082024-V.webp</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>45809.67502483061</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ASUS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Portátil Asus Vivobook X1502 Ci5-12500h 24gb Ssd512 Fhd15.6 color Quiet Blue</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/portatil-asus-vivobook-x1502-ci5-12500h-24gb-ssd512-fhd156-color-quiet-blue/p/MCO47191661?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO47191661&amp;position=5&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1569451947&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1929900</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2249000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>14% OFF</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>45809.67502484108</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LENOVO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lenovo Ideapad 1 Ip 1 15igl7 Intel Celeron N4020 15,6 Pulgadas 8 GB Ram</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/lenovo-ideapad-1-ip-1-15igl7-intel-celeron-n4020-156-pulgadas-8-gb-ram/p/MCO40332473?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO40332473&amp;position=18&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO2864083698&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1016900</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1500000</v>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>32% OFF</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Envío gratis</t>
-        </is>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>45809.67502484915</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Msi Cyborg 14 A13vf I7 16gb 512gb Ssd Rtx 4060 8gb Color Negro</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/msi-cyborg-14-a13vf-i7-16gb-512gb-ssd-rtx-4060-8gb-color-negro/p/MCO45076522?highlight=false&amp;headerTopBrand=true#polycard_client=search-nordic&amp;searchVariation=MCO45076522&amp;position=10&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1547623157&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4653900</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6999000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>33% OFF</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>45809.67502485745</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Potátil Portátil 14-dq0533la 14 8gb De Ram - 256gb Ssd - Intel Celeron</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=72GdK%2BpbrTFTM7i1sgjMu%2BbDsZwimgIVsgEMaqQVM80u2lSxiPxIp49lAD5FzvvX7tw%2B3WjmLZh4n%2BWEsTFcMPGWatgq50tuIi838LaR5oQJV5CEEvHbnKXPQACchyTHH0vjIO1%2Fj5c%2FXsO3bZMNq840pE4vh0ds%2Bd%2FwnVC79v072kXMRCGv3qHwC7U14OLGxP1MhOY85quB4Dd%2BoCzJ%2BVTsoBR7e70znoJTiR9qZUrKLyP%2BGL151fg2q%2FjTPcpe0EOWnfesuWGnIbRJ4UtBsHEOeSTUxpPqZKHMg8VjCEq4SmLvT%2BPRSReQB8aIUXznqFgDkSM1AE8omkj%2Fb%2FzxOs6KhMnCGKwZieGHEq6Q1rlE7c5VoFZGbp%2BOdt4PoLgaaqkzDbXOMhYOjXfdXrGgIzF6REZoUczzadV4ktrUlWshAxhwNxeakqcHnzwOFSCVPS4WrphjKzsUv3e3FIITEW1ZLpH%2BijyDAUSqj5BtIwnqZLC0aEfBTEKF086b3De50nkyz%2F1VJd4r2IhpVNLFE3P9mFqfBECnPRa1w%2Bj5TFMNuAMTPGDAZf%2Bp3f9QJMQ%2FrkuqXUtGmXqBcvaJSVoEKarvtyQY9iM9eRVEJGSve0Zvgw66yjF5rAZJXpCXH%2F0SuJqfrP1GZxnDkpeEMHfVYia4j959bA8TrP7ccIlaC37VeVRdDu%2F0329FzL07pGhmr0ABaZML9QGaZrqN7NpZPtdHai42qP5%2BxTxoA%2FgYEARxTAs3Y6XqVCueecJgOI7oc3f14YbulsBtatYNP%2Br%2FoKaJyI184MA5kvfmfDdC2Bfg12W8N6szceKHTo%2FthMXp4IoCP5VQNEK2vH5W%2FqMiPyumd%2FHlHpTXOTabOSyRlb%2BoYDSe4IzEy9SXmvrjE3GZPQi6T7ncDaOr3nL2yy%2BCUGFcYS4jRoUHT7Dr6RSMXBuSjuKMlIz5m2KgbW11LobjxwwP6xE%3D&amp;highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1547113619&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>919900</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1185375</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>22% OFF</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>45809.67502486529</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Portátil Hp 15-fd0026la Intel Core I3 8gb Ram 512gb Ssd</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=QHVRSkMapUYFd0MUsUJK5vva3fHEv%2FyYutnoyKQ309KPVo9qt3PSZ7ic6AU77nHcQz1SOsZVpaNDaqoo3MEy5TX%2Fx6omSlMudceAjcJe7TmVnVv6qgMEKiHF92%2FNwkqZ%2Fj%2FdQYtnH1YCcqK25LLkuC7M8zRZxibPMDqHhDa41LfQzT8c%2Fc2j3NZeddotr4mnhO%2FeiAgvZxsOVd0hkyHjXT6CpYL%2F7XgQFZsNyy%2Fomo3zxEpuqOyS3EuDTHF6K%2FM3k0hGvJK%2BS883r2s0w8NeHtjKUOh9ZDqR7cQneLG4ZVt4OwK51xKgfhII%2BzeCagUquSMbAp76%2FsgtCerLRz9BCuEE0PglxAd%2BjIr3MUL0%2Bgj5YJiP1EmHtBPGfqAY2mHskvzbW06do8Pjn%2BdFMX%2Fea8iyWi3OGOvq0O928uulkF5odhWAmKQcPvs5ZdHf3%2BnV0jb8WXXihcMGhQrADvxvEQH51JoKXOjYkgESygc010gYtqqzT3MiJs9RF%2FWpQr5CgHALRbn32vWyekuFqEFHmObrxqP%2B2mk25JoOhUWUdDpR9saNu0vKbpY8PWF1vyCe3mHfg9nILLA%2FWvCLLxP9da%2FPPyFYxZy%2FxjxaedElM9ABbpyy%2BtCcF7zXQlMoSWf7tTHpbaIhaW6sl4zv%2BsZiLd10R065djXFACsM7VKfZakLbHc0MwB%2FGgyi2RPCmVYd%2Fm5lu4XsHOCpLOCE3ApQF4LXLw6LVwxxpVpuLZb2E5zJRyJ0G9gt5xhE%2Bt1AFun%2BZBBd0X3oyTreYtHLOngjGLwPgPc1GdxghV%2B9wgeQ0zs0dm55nlM6w6DhGNJiRM6uQrAERZrHAAowzsKOY2ELq0Tz0lILYMyZxit0AxnKuccqHqrKCkl7iXonFO5zniizKB87r%2F%2B7DyxH%2B%2FtmdJ%2FoSMSeOcbPA%2BRGQ0Hgxz91UJBNRCeoO0ZHBzk0j4oq&amp;highlight=false&amp;headerTopBrand=true#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO2878894100&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2499900</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>45809.67502487299</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ASUS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Portátil Asus X1605za-mb644 Intel Corei5-12500h 16gb Ram Disco Solido 512ssd 16 Fhd Endless</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/portatil-asus-x1605za-mb644-intel-corei5-12500h-16gb-ram-disco-solido-512ssd-16-fhd-endless/p/MCO32161065?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO32161065&amp;position=3&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1523840021&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2029900</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>45809.67502488061</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ASUS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Portatil Asus E1504fa-nj474 Ryzen 5-7520u Ram 16gb Ssd 512gb Color Negro</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/portatil-asus-e1504fa-nj474-ryzen-5-7520u-ram-16gb-ssd-512gb-color-negro/p/MCO23498360?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO23498360&amp;position=14&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1541876389&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1725640</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1988778</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>13% OFF</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>4.8</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>343</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>413</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
         </is>
       </c>
-      <c r="L5" s="2" t="n">
-        <v>45809.63902662089</v>
+      <c r="M10" s="2" t="n">
+        <v>45809.67502488814</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>APPLE</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MacBook Air 13.6 M2 256 GB SSD 16 GB Ram Z160000au C/ Nota</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/macbook-air-136-m2-256-gb-ssd-16-gb-ram-z160000au-c-nota/p/MCO26602331?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO26602331&amp;position=8&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO2813970572&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4299299</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5057999</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>15% OFF</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>45809.67502489956</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Portátil HP 15-fd0065la Intel Core i5 16 GB 1 TB SSD 15.6" FHD Windows 11 Home</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=DGWR%2F%2Fegp7TdyCwhdw99a44O2oQgggn7VIYlmeQwtLg8VC08255MGlgaOJG9lbdJKyvhyvI7V5q1aLrsqe%2F4FmXlVusxQNzjHGFm5g0X44I9Dsb6kLzzhEiV4yyhD5iaunlUQefJHzTinDxyR0JqlbymbdlaJx4YYa%2FCdP4FSZgW409zFcLfSsXtpptnSgdJFrIwp86aGz9Uu%2Bd0iXBWcFs6tNefITwdYXIRpyNP1owqQcRMO1yu3x9MLyRXPUjvhwX5W%2ByYCjVFRzjY44o32cMJ1gFNlR5T7n%2BmX84DfqkNTgQkajcL1C4mjGHTtQF%2FhRsBBtUHfcGL0CNVwdGFMTRKj5OsAaex3wfqGTyl8gZ3yMZ3pWHT09upQ8aMymNrlLhYhZNGh6344jbKgSuTxWz2ICbIbPW6fv04fvzdEoEPzoovJO2RozxZhEDGCY0O7OLEkNqLcflDp7pVi2wf3VlmPLVEDFnwMLy1bXZr9kDNHjaskWf88CcTmrMhD3PUgyRWr7K82XAxD7KbQYCmIHWPrqh2tUpU7KUwtNFobF%2FxotC0yF3rHJOEkjYXg2NMxAt2i%2BuCNwQuC8vDNqSnOtqEemigcV%2BS5EvbSJq3wASgw%2BMwI3E4%2BGqWdMjBucyXDOCdLx3dHvUpWfjgAS28SQsLSS1Ibhp3FpUgUelSHlIeeD%2Fury1BdslGa%2F5tx3q95QSGQrmVaiIsNDTuMEc7QhT0%2F0sdRRw3O7tlRj8e54P5EF6Jr%2BnrIjBT3EIsDDDo2vl4XHq6zTCyg2O2ZVGDf0K%2BDoZiDzpwyBm1E5eBuYO2uR9R2NjL91NqgaFVTKAIyOUdFX3x8ou7kmR5%2BlzbnrqYk9tZiILIOGAOgZ7o1oVT4qIHvzVExprTu2ZXRN5kJKv7UdzoUn4k6mdexHYG83G4d810%2BP2GcSek7%2Fu7AWabbdd3B%2FMmqC3tYtvaGMeF6ySSBG9rpBVymR946CS9Jt0rJlOf%2BQ%3D%3D&amp;highlight=false&amp;headerTopBrand=true#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1575797741&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2500939</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4099900</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>39% OFF</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>45809.67502491106</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Portátil Hp 14-em0009la R5 Ram 16gb 512gb Ssd</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=Ui85GGnE61myuhHJSIj0W1rPFgRVo6zApHFyKPftQVLNje9pXasbLvsWHLlFW4MhTRm9ZVeNOrB%2BngajZe8OrVI%2B4nE0K755kqb%2FPICRTgQQEeui%2Bb4erSxuD2POwCn3AK3hEr8UWhN1sDL0bZVt3MHfDnIuEec5gqyaVVoILB185p2wzrsbuOqLXNnou%2FqXgegJBYuVpWHMCXM0%2Fmg1PuPIXlQpqw8Xcppha0utEmiCoygIzCgI51Q%2F3LcsU3Ke9%2BdgGo6cMQ7ACngoSaKyT6l1mvp9EtTdOgAno9qK738ZPQZdqyck1rzjCe6M8v0ViWqCcCkhXpeHhw6ho1tdX3EQU%2B4WDS2OR2gXBKcsK3S3LNiZATtjJxNq2PUOCYaqC9SG1DStQvFywgjF3mM5dLviPgGkFxg9BWvFd9Aa0T47iQZ0hL3L58W0ZzZvjQrHhO93f22Pa4QqGAlTf5BDjt5HY1TCUZclgyI9ARL7IwRLQ5EB4K%2B4J6JGRi%2BWO8jL8U00tNAUDKg%2FmoSvXhNTbdxhaiYyD0mnbxF4wPe5%2BURIe21utXPEWRO69wxZjtT4YWLb0XPYhA7X17bVJq83OmwciLx2fcUb6R%2FvvxVGY0eafDscgnAOnr1ACE08qK0jz5Y4JeSnOh%2Fypcc0Y%2BKB3ENzXJTzKcthsQxXozKrDfDlJIEMVhJzKyi9YpVJ6o8XtAVaF4G5UldPvlRAoUSihWWZaLyHQyICEtWwcaC3h0HuXHOBx0WI%2FFP1EzmtqhecdHo%2Fo1Mel7XBq77HH1ohe37Ti7LTX5Bd2sARF6avfVwT0KF6RDZ%2Fk6U5H9PExFYXGEHR0LBIuGYLgja7vux3NZBgrdEetEylgbMKRvINLvr3azROENAA9eOKRGaOZQuZZEW7rT2CI%2FmkP88zDBvjBNNokaY26yoO0Ox5oAqw8cfh7C8Q&amp;highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO2503419712&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1770900</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2248125</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>21% OFF</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>45809.67502491979</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Notebook 15,6 Hp 250 G9 Intel Celeron 8 Gb Ram 256 Gb Ssd Color Negro</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/notebook-156-hp-250-g9-intel-celeron-8-gb-ram-256-gb-ssd-color-negro/p/MCO24443216?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO24443216&amp;position=21&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1479324193&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>902003</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1094000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>17% OFF</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>45809.67502492775</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Notebook Hp 245 G10 R3 7330u 512gb Ssd 8gb Ram Windows 11 Ho</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/notebook-hp-245-g10-r3-7330u-512gb-ssd-8gb-ram-windows-11-ho/p/MCO39243137?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO39243137&amp;backend_model=search-backend&amp;position=26&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1547113843&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1259900</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1621375</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>22% OFF</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>45809.67502493539</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Portatil Hp 12ava Gen Intel I3 1215u Ssd 512gb Ram 8gb Color Plateado</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/portatil-hp-12ava-gen-intel-i3-1215u-ssd-512gb-ram-8gb-color-plateado/p/MCO29272690?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO29272690&amp;backend_model=search-backend&amp;position=4&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1507088307&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1458900</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1853000</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>21% OFF</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>45809.67502494298</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Portátil 2 en 1 HP Pavilion x360 14-ek1011la Intel Core i5 8 GB RAM 512 GB SSD Windows 11 Home 14" Pantalla táctil FHD</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=2isFgknxOdut9wXlQP0iITpWbs1sARTKTrjHXi%2FMHoczuv2WAdftWVdjPOA74d0RTmEsftMgUsX%2FMM9WXr3j6V%2BAGQ5AG0mIUS5JeEpPBgOTLLj9j8smzhuqpQBQjNLyVlDeYKF07dG00UJvY8tW03dkej5aTdZXNrfk3PmFZbK%2BqlohQF5UEMj%2FIOyKa%2FvLqYa6hoU6ep2lvqBBSycW%2BfOxLR%2Flue%2BMYWuzgRUO3h5oDGDSl7nsWFzlfHPZwOEL%2Brb5r1rvmQo9Owa6Q%2BZ%2FAwSwNAKAcrHhGUR5p7i3Tu35wg5iYCN95AbBBaYXr4nWFHJd9aREV%2B8eyeMpRLOmgihamWbGJfx9kbCvA3ihk8O%2ByWg7SFx5vzw5iA4j5C5uIyyJakoIXATauCzp3YpvOU4Lv%2FzfmwebiBWkcGO%2FpSNO5xV%2FsS4uUp2TekeO7nEfl6FF6Q8xYisLj8K5%2FLruUauzWaCcd6r0EOLnWcMT1VYHzWFp%2FDPpRD%2FM%2BwCTJyD0HLyRaq9o3rX%2BT2OqetnPt4fohuMeVwsb9neAnKOmZ%2B1%2BHU0aIUt%2FA3CPxA64TMmcBTWBUCXloFCybUI9ecZgtWWls40ZEJ6gGaTQSxtaMWf3ZXupuSMAtSGBF3B56W4g5CrbJQHCo1mXQudc%2B6HoSihb1jHSNpKQ05CmNdJZXA2lMG6KyWls2mkEatxNrm100RTtxcZjwjQL%2BRdsR3eo7RuAfrRnkuOwo5ghO%2F9lIq8TVPTszdCJZ6%2B9roXQXQKSqZlExdB2iI1X2ktZkJsAJu96%2BJtFu5U1DSZ%2FHj%2F660BTG0AFaY2iO75lVXam8o6kRrsJgYQlXUz7egDl%2By12SqXEPGquC1RhDls2Vkx9PXBL60XshaTSv8NAPFP6odNk%2BHBUZPdkZ%2FHXBR4dI%2FfemcTtW0L7djFRtZhGfkgQXlOBoyDkaWGqw%2FnF4Vea1ip7RDKPokO%2BIRd752yYsaCXTln0D6jU3vNsoG%2BMiz76COhTZvFRVzbQeb13%2B0BXls2OHFOjgIFgoi4GDdSGTQ%3D%3D&amp;highlight=false&amp;headerTopBrand=true#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO2859705258&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2519937</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3999900</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>37% OFF</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>45809.67502495056</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Portátil HP 15-fc0031la AMD Ryzen 7 16 GB RAM 1 TB SSD 15.6" FHD Windows 11 Home</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=JpCyesSU7FvVnsZ5%2BL%2BzJrom0whIfM9UkilyAkynRPaHNJZmxB99RszVeXnjGIOckALEtIxHh1slZJmJJZoKnNuK5T3uMKFO2fcm3m64QAFDQ9FAFbaB6WT8kFxDzwsYdlwgcNGfhxb700tBs7NQYUX5EX81d6toSPxUzBuoudpAdd73klj7wdkOxsXIBiBduaoOFVwrFMjPui3aDRtdTlfPVgxuMdb6QizMiJWoQL5yg%2BF9SNhtPC7JQuvdGonOsHYJZCrdn%2FacVfMU0rKQQiSAO940mnjoCVoI5e%2BgGu3qnPiZL4TiiZmLWhu8BfionVN263LyNNKcLXtyfzs3rLR8Q25zjk7fIx%2B%2BDOwEEhVyz93nQpLfRyv7o65GvS4mBp5QHYMrX%2BOeDGHZXJO7dC%2Fr68BhGLKnGCvPybClst%2Brq%2BAKwgzeaFF%2Bw5qB4P0zbnzRDg3UTy0tWaJ0psAyyfnH6zS6rOQaigRFvHc%2BaJwaj3z0IONiFeRWi%2BN%2BG1GeecLJQ5Ijf0q2cU7UnVDWH2vZGmkP7WeSIlphoeTggF6D8Bqt%2F44rx2Kn8KGZAx1YM%2Buu4SD34aS%2FsomMNGRnEqUgkB4cnXNAKLAjATKp%2BwGGf8DWBGRxElZ%2FPkzlI7gfKDJyeKG%2BPw8yuMnt%2FvtZ3D0DwkEhj6xZUBksUANEVmwfzk6jxBCHoCfCcxnHLsLd%2FZ%2BqDlRr8LDIQAwUHkmPOgELwi7y0ZGkEKStk0h0MYd0jnjbrev63gap47u4m5c%2FoeDhPyjZ5Iu3%2Fb6myKcEYq8cCOwlmNTwofIUOS8s1aBVwZSXmlKHI4gLMQbGT0tFb5%2FH11Z2ejFEq6FOp9Pgy9REGbBO%2BFIqmpf%2FqYQShEUhzLWeI02lc8Aei%2FVkPhA23v4Qk5kEpNvwwZT9JKOlrY1XBykOUEeSbZUfWluYetUgLeg%2FnpxvJ9omITuzni4YJONdH5MNBlRoeQqVG2vZzo1iTuarHA%3D%3D&amp;highlight=true&amp;headerTopBrand=true#polycard_client=search-nordic&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1575771851&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4099900</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>45809.67502495806</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LENOVO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Portatil Lenovo V14 Core I5-13420h 24gb 512gb Ssd Color Negro</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/portatil-lenovo-v14-core-i5-13420h-24gb-512gb-ssd-color-negro/p/MCO44279796?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO44279796&amp;position=13&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1587144125&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1900230</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2176667</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>12% OFF</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>45809.67502496565</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ASUS</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Portátil Asus Fa506nc Ryzen 5 7535hs Rtx3050 16gb 512gb 15.6 Color Negro</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/portatil-asus-fa506nc-ryzen-5-7535hs-rtx3050-16gb-512gb-156-color-negro/p/MCO45003983?highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO45003983&amp;position=9&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1544070727&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2975814</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3199800</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>7% OFF</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>45809.67502497309</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Potátil Portátil 14-dq0533la 14 8gb De Ram - 256gb Ssd - Intel Celeron</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/potatil-portatil-14-dq0533la-14-8gb-de-ram-256gb-ssd-intel-celeron/p/MCO43485439?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO43485439&amp;backend_model=search-backend&amp;position=27&amp;search_layout=stack&amp;type=product&amp;tracking_id=f57ed311-6736-4ff6-90fb-6463ca5135c1&amp;wid=MCO1547113619&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>919900</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1185375</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>22% OFF</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>45809.67502498048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar funcionalidad para obtener imágenes de alta calidad de productos en el scraper de MercadoLibre. Se actualiza la función `scrape_mercadolibre` para incluir la obtención de imágenes y se modifica la clase `ExcelHandler` para registrar las imágenes en el archivo Excel.
</commit_message>
<xml_diff>
--- a/productos_mercadolibre.xlsx
+++ b/productos_mercadolibre.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monitores" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="laptos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tablet" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="teclados" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2093,11 +2094,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Tablet Android 13 De Última Generación 2024, 128gb+16gb-512g</t>
@@ -2130,15 +2127,9 @@
       <c r="I2" t="b">
         <v>0</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -2151,7 +2142,7 @@
         </is>
       </c>
       <c r="N2" s="2" t="n">
-        <v>45809.67834955709</v>
+        <v>45809.67834956018</v>
       </c>
     </row>
     <row r="3">
@@ -2192,28 +2183,415 @@
       <c r="I3" t="b">
         <v>0</v>
       </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '14 may. 2025', 'contenido': 'Realmente pensado para los pequeños.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>45809.67834958334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tablet Xiaomi Redmi Pad Se 8gb 256gb Gris</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/tablet-xiaomi-redmi-pad-se-8gb-256gb-gris/p/MCO29219683?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO29219683&amp;position=4&amp;search_layout=stack&amp;type=product&amp;tracking_id=de599f53-e149-4e6e-87ca-312bb77ee567&amp;wid=MCO1567332181&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>709900</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1149900</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>38% OFF</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="K4" t="n">
+        <v>298</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '26 jul. 2024', 'contenido': 'La tablet es demasiado rápida, corre juegos con facilidad y su pantalla es muy buena. Le verdad me sorprendió lo bueno que corre los juegos y las aplicaciones.', 'votos_utiles': '13'}, {'calificacion': 5, 'fecha': '08 jun. 2024', 'contenido': 'Excelente compra. Una tablet de calidad,buena construcción e increíble apariencia. Definitivamente otro gran producto de xiaomi.', 'votos_utiles': '8'}, {'calificacion': 5, 'fecha': '29 ene. 2025', 'contenido': 'Súper me gustó mucho , apenas para lo que necesito 😊.', 'votos_utiles': '6'}, {'calificacion': 5, 'fecha': '30 dic. 2024', 'contenido': 'Genial.', 'votos_utiles': '3'}, {'calificacion': 5, 'fecha': '17 feb. 2025', 'contenido': '', 'votos_utiles': '3'}]</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>45809.67834959491</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LENOVO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tablet Lenovo Tab K11 4g Lte 8gb 128gb Teclado + Pen Color Luna Grey</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/tablet-lenovo-tab-k11-4g-lte-8gb-128gb-teclado-pen-color-luna-grey/p/MCO45442884?highlight=true&amp;headerTopBrand=true#polycard_client=search-nordic&amp;searchVariation=MCO45442884&amp;position=5&amp;search_layout=stack&amp;type=product&amp;tracking_id=de599f53-e149-4e6e-87ca-312bb77ee567&amp;wid=MCO1529700467&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1094900</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1899900</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>42% OFF</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '15 may. 2025', 'contenido': 'Exelente producto calidad precio. Lo recomiendo totalmente.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '08 may. 2025', 'contenido': 'Bonita y económica.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '30 abr. 2025', 'contenido': 'Muy buena y muy práctica.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '03 mar. 2025', 'contenido': 'Es muy buena.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '10 feb. 2025', 'contenido': 'Excelente!.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>45809.67834960648</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LENOVO</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tablet Lenovo M11 128gb 8gb Ram + Lapiz 10.9 Pulgadas Color Negro</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/tablet-lenovo-m11-128gb-8gb-ram-lapiz-109-pulgadas-color-negro/p/MCO36109372?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO36109372&amp;position=8&amp;search_layout=stack&amp;type=product&amp;tracking_id=de599f53-e149-4e6e-87ca-312bb77ee567&amp;wid=MCO1501072863&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>874900</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="K6" t="n">
+        <v>167</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '10 jun. 2024', 'contenido': 'Me parece muy bien por el precio pero se descarga muy rapido.', 'votos_utiles': '12'}, {'calificacion': 5, 'fecha': '03 sep. 2024', 'contenido': 'Increíble, muy buen precio, excelente calidad. Es rápida la pantalla es muy buena, buena carga, en uso continuo puede durar todo el día.', 'votos_utiles': '9'}, {'calificacion': 5, 'fecha': '26 nov. 2024', 'contenido': 'Vale totalmente la pena por su precio.', 'votos_utiles': '7'}, {'calificacion': 5, 'fecha': '09 may. 2025', 'contenido': 'Un producto, que respecto a la calidad precio, está muy bien.\nPuntos a favor:.\n1. Lapiz para trabajar, cumple perfectamente con la función, con una duracion de su bateria, aceptable, alrededor de una semana con trabajo constante.\n2. Tiene un buen sonido, claro, y con buenos decibeles, no es premium, claro está.\n3. Viene con un buen forro o cubierta, que ayuda a mantenerla seguro, y con mayor comodidad.\n4. Respecto a su software, está bien logrado, fluye con practicamente todo, obviamente no está hecha para jugar aplicativos mayormente exigente, pero para trabajos cotidianos, está excellent. Viene con un aplicativo didactico, para tomar apuntes, y hacer calculos, entre otras opciones.\nPuntos debiles:.\n1. La pantalla, puede mejorar un poco mas, no tiene la mayor iluminación, no es ultra hd, ni nada parecido.\n2. Las camaras no son para realizar videos, imagenes, o videollamadas respectivamente, tienen muy poca resolución, simplemente cumplen.\n3. La bateria si es su punto mas debil, dura muy poco, con trabajo constante, y hay que tener en cuenta, que su carga es lenta, se puede demorar 3 horas en cargar approx.\n4. Llevo alrededor de 6 meses utilizandola, y me ha presentado un par de fallas respecto al sonido, he tenido la obligación de reiniciarle, y se ha solucionado.\nBuen producto, para el que busque algo correcto a buen precio.', 'votos_utiles': '4'}, {'calificacion': 5, 'fecha': '02 dic. 2024', 'contenido': 'Excelente producto en relación precio/calidad. Ha cumplido en las tareas en que la he usado como edición de video y toma de apuntes. El lápiz funciona bastante bien.', 'votos_utiles': '3'}]</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>45809.67834960648</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>precio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>precio_anterior</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>descuento</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>envio</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>envio_gratis</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>envio_full</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>total_reviews</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>imagen</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>imagenes</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>opiniones</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_actualizacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Teclado Mecánico Inalámbrico Newmen Gm610 60% Rgb 61 Teclas</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=6gGtzBLavbK6QT%2FHNpbmv4xJiCt5aKMxBqNom0ChA44NtPEmuvAI%2Bd%2F6wZ5bJEEzHJr5DnaUPSSbXsA27RKEa9B2aGtGEO0TsJfkfy%2BAxjueSxf%2Bb63DYr8jbEaPbuHXO%2B5hpSgqQj9g65y8837ovhh%2FLr824TMjzjtbqPPd1LhEsdCYo22TnDqIeTtfDnpv%2FtmlNqz637XVhPscnSGmouUrSXmqrjeiCPDnf9KVlls8EDsrjF6s%2FERJT5%2BzF0fY%2BttMYUcQwgDnN1mOlZZlKQBr4sMtGrWiG8OFpv3c5EpaylXa%2FBdBvq0jhw70H0oSxSxvb5cuBpONRrhOyv4yPwuTc66azMz98G5fX8C7KZF7EeV99fWGhMOdqwMYvMam8gmrw2AZbdNRtAywmoN06LhUPPXLSsM5kUKroJuLUM3VAkVh5zRqQl%2FQIyXSGPcU5D0nva18v1VGvdIwqwfh0Ibf9JkqBEaIGeZn%2B40QC5od%2Bjf0ozYJOAVdaA8WvEwj%2BOWRrMKdheFNCYVp7FSXsnuyEEYCYT8c%2BbHZ9DLdBMTVctfuHGmPhsO06wVqqTA5Y9fxJHdJBiSPDU5UmhG7ISvZHMV8sxffBRRUzlfKORPzCa8A6pK5AQQRfjBoRFsl6wSRBx8J4hW%2BkAQSay2F6gt1pVQXmsmhXspXlNdWknhJY2OhJ9MCfhbJ91LuskxMN00efWb6svoHLy7UXfl6CJqma5A6SUsiBa%2BKC%2FErjG6jRQrzTjmECxwEUl9YdmtjbYMdwwtDSGKR6Q5JunQwTqCRCplf%2FAWojZHys7g2isSZ2GvCIsWBEAbpoUVJcToj87qK1lwTBs6zEde6g8iRNugxlwcuSepuSFkKENccA3ZAs4Y3wZOlkfOr2xC%2BxxbvOb00Ed6IwFkjIrpK0lfUyePM9tiooSvD8Imm2h7b8Ayff8r0mq9HUCBj%2FrCUw2tA&amp;highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO2573729598&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>144415</v>
+      </c>
+      <c r="E2" t="n">
+        <v>169900</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>15% OFF</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_940676-MLU77417106611_072024-V.webp</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_940676-MLU77417106611_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_987647-MLA82113006950_022025-F.jpg', 'https://http2.mlstatic.com/D_NQ_NP_2X_756226-MLU78420919739_082024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_708773-MLA84456438700_052025-F.webp']</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '13 sep. 2024', 'contenido': 'Es un producto hermoso, recomiendo instalar el firmware desde la pagina oficial según como indica el manual, arregla un conflicto con varias teclas. También recomiendo poner el idioma del teclado en el pc como ingles us para que no hayan problemas. Siguiendo los pasos que les acabo de mencionar el producto es maravilloso. Lo mejor que se puede conseguir calidad precio. Pdta toca acostumbrarse a dar un comando para usar las flechas y no tiene la tecla ñ.', 'votos_utiles': '8'}, {'calificacion': 5, 'fecha': '09 oct. 2024', 'contenido': 'Extremadamente bueno, una compra que uno no se arrepiente lo recomiendo.', 'votos_utiles': '3'}, {'calificacion': 5, 'fecha': '09 dic. 2024', 'contenido': 'Me gustó, las orientaciones de los usuarios sirvieron mucho … fácil de instalar , dejarlo en opción inglés y para la tilde o ñ se coloca en español … las luces del teclado súper , recomendado !!!.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '31 may. 2025', 'contenido': 'El teclado muy bueno para su precio. La verdad no estaba esperando mucho sino que funcionara bien y fuera cómodo al tacto. A la final ha superado mis expectativas. Muchas gracias.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '27 may. 2025', 'contenido': '', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>45809.68173760112</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Teclado Gamer Mecanico En Español Retroiluminado Con Cable Usb Xtrike Me Gk988 Para Computadora Pc Con Luz</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=f%2F2y0a41zS%2FCSk3LHoy1FmCIOd3IXjkIc4zrxquwe11mnEs31DNrGs4s5WGrbswIcV9mcJMF42%2F%2FNXENqgyu%2FlQzWscGtdgGm5pc%2B4n1Mt2puld%2B2kCs6YlAYLN7ouABMzMjt%2F0MYeuzXcRO5DM9XfBU8IqWp9tAW3BFhiBnyl8%2FEcst8TuhHvi2lI%2BYgB8c9M0z98WMPpnCrYD80Sdi2iGnAb4xjTGp5qvj7foeTG%2FxBA6vSiEBLE7x2UlQ5Ml3lWzVVIV4vKuU%2BhwsQeqCbXkZF352uL4OCafSvy3oYmZxbvVKS4JXJUP3BVDLkKpIWr3Xqhn3LVG6gKoQAPlvIOQsjYpRCm6cg1kks2jGkl8Ww2owqqEFRTdb7EDuWwfZx8mOZeMIAZ4Hg1IxyPhjLXQ%2FdkUJky0iTAWe1OFTOxT1evOPhkW3GPSk721VWfZi84JlxLNJM8j87%2BqEhX5aO7rSB662JU%2BxI9EfURh6WoqdG19xLTWj4WcEVGELrCM7oYoYwyBxEFcuVP9iUiljdTIuHScEneuLOOWeyvSpZ2NoUOEUAikCrQW7X%2FiDWTIZgdyzRusJ%2BIJx3BpsuUWAEbWZoOIQMXAztgzgmtR1AELcUYbBQ7vV9HSAwbZsoj2AJxmLku7N6X1okzof6Fpbdtwe9Hbopr1YSWTf1zWCM6IwMRXXbmsXBZtKQfwi4Pk6KJGj4HXWS02mdU5DGAOgcok5du2bgnYgo8NMgHPAOWvmmlcnd85ssCEg9fKKkcMjGWbETWPSh7xiDsGnSXXwTNNXK8GMp94WkD8bjcDXGq8mL8n1bt717kIG8rEnssoov07dc1xhHx0%2FlVtteyt8LTFvmsiiMpKZzXqV3he5op527UBvZsM2U9QaHewKaBvicFrw%2FTMjgedgArbI43oicXIeLU61Oshp5Tg8FOSkOaz2yD%2FKLgOF86LVMyp%2FsVQ1vs%2FBsIAonsMEK38835kntHbMho%2FMJb2hEARHJajFWEaHs7iZ0y9oh%2Fse2pcNlrw%3D&amp;highlight=true&amp;headerTopBrand=true#polycard_client=search-nordic&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO1560382775&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>104900</v>
+      </c>
+      <c r="E3" t="n">
+        <v>149900</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>30% OFF</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>19</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_973583-MLA83472189647_042025-V.webp</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[{'calificacion': 5, 'fecha': '14 may. 2025', 'contenido': 'Realmente pensado para los pequeños.', 'votos_utiles': '0'}]</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>45809.67834958383</v>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_973583-MLA83472189647_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_833541-MLA80825743061_112024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_820938-MLA80563766270_112024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_760094-MLA80563785792_112024-F.webp']</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '01 may. 2025', 'contenido': 'Contento con el producto.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '28 abr. 2025', 'contenido': 'Es una buena opción por el precio, cumple con lo que promete perfectamente, se siente de buena calidad y al responde bien, recomendado.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '31 may. 2025', 'contenido': 'Bastante bien calidad precio:) lo recomiendo!(es algo ruidoso) perfecto para competitivo.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '23 may. 2025', 'contenido': 'Se ve excelente, me gusto mucho.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '22 may. 2025', 'contenido': 'Cumple con todo. Muy buen producto.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>45809.6817376265</v>
       </c>
     </row>
     <row r="4">
@@ -2224,23 +2602,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tablet Xiaomi Redmi Pad Se 8gb 256gb Gris</t>
+          <t>Teclado gamer Redragon Kumara QWERTY Outemu Red español España color negro con luz rainbow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.mercadolibre.com.co/tablet-xiaomi-redmi-pad-se-8gb-256gb-gris/p/MCO29219683?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO29219683&amp;position=4&amp;search_layout=stack&amp;type=product&amp;tracking_id=de599f53-e149-4e6e-87ca-312bb77ee567&amp;wid=MCO1567332181&amp;sid=search</t>
+          <t>https://www.mercadolibre.com.co/teclado-gamer-redragon-kumara-qwerty-outemu-red-espanol-espana-color-negro-con-luz-rainbow/p/MCO19518470?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO19518470&amp;position=3&amp;search_layout=stack&amp;type=product&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO1347087050&amp;sid=search</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>709900</v>
+        <v>190900</v>
       </c>
       <c r="E4" t="n">
-        <v>1149900</v>
+        <v>199900</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>38% OFF</t>
+          <t>4% OFF</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2261,7 +2639,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>298</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2271,38 +2649,43 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>[{'calificacion': 5, 'fecha': '26 jul. 2024', 'contenido': 'La tablet es demasiado rápida, corre juegos con facilidad y su pantalla es muy buena. Le verdad me sorprendió lo bueno que corre los juegos y las aplicaciones.', 'votos_utiles': '13'}, {'calificacion': 5, 'fecha': '08 jun. 2024', 'contenido': 'Excelente compra. Una tablet de calidad,buena construcción e increíble apariencia. Definitivamente otro gran producto de xiaomi.', 'votos_utiles': '8'}, {'calificacion': 5, 'fecha': '29 ene. 2025', 'contenido': 'Súper me gustó mucho , apenas para lo que necesito 😊.', 'votos_utiles': '6'}, {'calificacion': 5, 'fecha': '30 dic. 2024', 'contenido': 'Genial.', 'votos_utiles': '3'}, {'calificacion': 5, 'fecha': '17 feb. 2025', 'contenido': '', 'votos_utiles': '3'}]</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>45809.67834959479</v>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_636746-MLA52350707355_112022-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_913394-MLA52350707356_112022-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_994079-MLA52350716250_112022-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_912260-MLA52350716251_112022-F.webp']</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '08 may. 2021', 'contenido': 'Panas yo lo veo bien xd, tal vez sería mejor si las luces fueran más brillantes pero de resto llevo 1 mes con el y todo gucci, todo bien todo correcto además me regalaron unas teclas de cambio :) uwu.', 'votos_utiles': '56'}, {'calificacion': 5, 'fecha': '14 jun. 2023', 'contenido': 'Me encantó llevo más o menos 1 año con el producto y no ha presentado problemas, se escucha bien y se ve bien 😎.', 'votos_utiles': '35'}, {'calificacion': 5, 'fecha': '17 ago. 2023', 'contenido': 'El producto es bastante bueno en calidad-precio; cositas que no me acabaron de gustar, pero que son de menor importancia para mi son que algunas partes de las teclas (ej. Bloq mayús) que no se iluminan completamente, no tienen switches brown para comprarlos con el teclado, las patitas de goma antideslizantes no son las mejores, el teclado se tambalea un poquito aunque no se si es mi escritorio o el teclado (con el manual en una esquina se arreglo), de resto es un buen teclado, los materiales en acero para la placa y el "plástico reforzado" están decentes, el cable no es mayado, pero tiene el conector usb en oro chapado (creo que así se le dice xd), es hotswap, por si le quieren poner otros switches, la retroiluminación es decente y algo que me parece vital, pero no tiene, es que el conector no es removible, en general lo recomiendo si no hay mucho dinero para gastar y cuando ya se tenga el set-up bien armado cambiar el teclado o dejarlo.', 'votos_utiles': '12'}, {'calificacion': 5, 'fecha': '26 jun. 2021', 'contenido': 'Bastante bueno, la verdad tanto el tacto como el sonido me gustó demasiado, es bastante bonito gracias al color rojo que arroja el teclado por defecto, es algo pesado lo que hace que sea difícil moverlo sin querer lo cuál es genial, es tenkeyless lo que hace que te quede bastante más espacio del que uno cree que le va a quedar y la verdad estoy tratando de hacer la reseña larga porque es bastante cómodo escribir con este teclado.', 'votos_utiles': '10'}, {'calificacion': 5, 'fecha': '07 sep. 2023', 'contenido': 'Lo recomiendo, excelente producto ☺️ buen material.', 'votos_utiles': '7'}]</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>45809.6817376367</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tablet Lenovo Tab K11 4g Lte 8gb 128gb Teclado + Pen Color Luna Grey</t>
+          <t>Teclado gamer Redragon Kumara QWERTY Outemu Red español latinoamérica color negro con luz RGB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.mercadolibre.com.co/tablet-lenovo-tab-k11-4g-lte-8gb-128gb-teclado-pen-color-luna-grey/p/MCO45442884?highlight=true&amp;headerTopBrand=true#polycard_client=search-nordic&amp;searchVariation=MCO45442884&amp;position=5&amp;search_layout=stack&amp;type=product&amp;tracking_id=de599f53-e149-4e6e-87ca-312bb77ee567&amp;wid=MCO1529700467&amp;sid=search</t>
+          <t>https://www.mercadolibre.com.co/teclado-gamer-redragon-kumara-qwerty-outemu-red-espanol-latinoamerica-color-negro-con-luz-rgb/p/MCO19472215?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO19472215&amp;position=4&amp;search_layout=stack&amp;type=product&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO1483729915&amp;sid=search</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1094900</v>
+        <v>190900</v>
       </c>
       <c r="E5" t="n">
-        <v>1899900</v>
+        <v>198000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>42% OFF</t>
+          <t>3% OFF</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2318,12 +2701,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -2333,31 +2716,36 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[{'calificacion': 5, 'fecha': '15 may. 2025', 'contenido': 'Exelente producto calidad precio. Lo recomiendo totalmente.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '08 may. 2025', 'contenido': 'Bonita y económica.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '30 abr. 2025', 'contenido': 'Muy buena y muy práctica.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '03 mar. 2025', 'contenido': 'Es muy buena.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '10 feb. 2025', 'contenido': 'Excelente!.', 'votos_utiles': '0'}]</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="n">
-        <v>45809.67834960301</v>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_864807-MLA77594879101_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_625461-MLA75686545678_042024-F.jpg', 'https://http2.mlstatic.com/D_NQ_NP_2X_867951-MLA77594879095_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_750884-MLA77378571910_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_845414-MLA77378789172_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_901847-MLA77378571898_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_804807-MLA77378808744_072024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_909019-MLA74488153000_022024-F.jpg']</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '08 may. 2021', 'contenido': 'Panas yo lo veo bien xd, tal vez sería mejor si las luces fueran más brillantes pero de resto llevo 1 mes con el y todo gucci, todo bien todo correcto además me regalaron unas teclas de cambio :) uwu.', 'votos_utiles': '56'}, {'calificacion': 5, 'fecha': '14 jun. 2023', 'contenido': 'Me encantó llevo más o menos 1 año con el producto y no ha presentado problemas, se escucha bien y se ve bien 😎.', 'votos_utiles': '35'}, {'calificacion': 5, 'fecha': '17 ago. 2023', 'contenido': 'El producto es bastante bueno en calidad-precio; cositas que no me acabaron de gustar, pero que son de menor importancia para mi son que algunas partes de las teclas (ej. Bloq mayús) que no se iluminan completamente, no tienen switches brown para comprarlos con el teclado, las patitas de goma antideslizantes no son las mejores, el teclado se tambalea un poquito aunque no se si es mi escritorio o el teclado (con el manual en una esquina se arreglo), de resto es un buen teclado, los materiales en acero para la placa y el "plástico reforzado" están decentes, el cable no es mayado, pero tiene el conector usb en oro chapado (creo que así se le dice xd), es hotswap, por si le quieren poner otros switches, la retroiluminación es decente y algo que me parece vital, pero no tiene, es que el conector no es removible, en general lo recomiendo si no hay mucho dinero para gastar y cuando ya se tenga el set-up bien armado cambiar el teclado o dejarlo.', 'votos_utiles': '12'}, {'calificacion': 5, 'fecha': '26 jun. 2021', 'contenido': 'Bastante bueno, la verdad tanto el tacto como el sonido me gustó demasiado, es bastante bonito gracias al color rojo que arroja el teclado por defecto, es algo pesado lo que hace que sea difícil moverlo sin querer lo cuál es genial, es tenkeyless lo que hace que te quede bastante más espacio del que uno cree que le va a quedar y la verdad estoy tratando de hacer la reseña larga porque es bastante cómodo escribir con este teclado.', 'votos_utiles': '10'}, {'calificacion': 5, 'fecha': '07 sep. 2023', 'contenido': 'Lo recomiendo, excelente producto ☺️ buen material.', 'votos_utiles': '7'}]</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>45809.68173764625</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LENOVO</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tablet Lenovo M11 128gb 8gb Ram + Lapiz 10.9 Pulgadas Color Negro</t>
+          <t>Teclado gamer Redragon Mitra QWERTY Outemu Blue español latinoamérica color negro con luz RGB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.mercadolibre.com.co/tablet-lenovo-m11-128gb-8gb-ram-lapiz-109-pulgadas-color-negro/p/MCO36109372?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO36109372&amp;position=8&amp;search_layout=stack&amp;type=product&amp;tracking_id=de599f53-e149-4e6e-87ca-312bb77ee567&amp;wid=MCO1501072863&amp;sid=search</t>
+          <t>https://www.mercadolibre.com.co/teclado-gamer-redragon-mitra-qwerty-outemu-blue-espanol-latinoamerica-color-negro-con-luz-rgb/p/MCO15079758?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO15079758&amp;position=9&amp;search_layout=stack&amp;type=product&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO1505508309&amp;sid=search</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>874900</v>
+        <v>279900</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -2385,7 +2773,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2395,11 +2783,351 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>[{'calificacion': 5, 'fecha': '10 jun. 2024', 'contenido': 'Me parece muy bien por el precio pero se descarga muy rapido.', 'votos_utiles': '12'}, {'calificacion': 5, 'fecha': '03 sep. 2024', 'contenido': 'Increíble, muy buen precio, excelente calidad. Es rápida la pantalla es muy buena, buena carga, en uso continuo puede durar todo el día.', 'votos_utiles': '9'}, {'calificacion': 5, 'fecha': '26 nov. 2024', 'contenido': 'Vale totalmente la pena por su precio.', 'votos_utiles': '7'}, {'calificacion': 5, 'fecha': '09 may. 2025', 'contenido': 'Un producto, que respecto a la calidad precio, está muy bien.\nPuntos a favor:.\n1. Lapiz para trabajar, cumple perfectamente con la función, con una duracion de su bateria, aceptable, alrededor de una semana con trabajo constante.\n2. Tiene un buen sonido, claro, y con buenos decibeles, no es premium, claro está.\n3. Viene con un buen forro o cubierta, que ayuda a mantenerla seguro, y con mayor comodidad.\n4. Respecto a su software, está bien logrado, fluye con practicamente todo, obviamente no está hecha para jugar aplicativos mayormente exigente, pero para trabajos cotidianos, está excellent. Viene con un aplicativo didactico, para tomar apuntes, y hacer calculos, entre otras opciones.\nPuntos debiles:.\n1. La pantalla, puede mejorar un poco mas, no tiene la mayor iluminación, no es ultra hd, ni nada parecido.\n2. Las camaras no son para realizar videos, imagenes, o videollamadas respectivamente, tienen muy poca resolución, simplemente cumplen.\n3. La bateria si es su punto mas debil, dura muy poco, con trabajo constante, y hay que tener en cuenta, que su carga es lenta, se puede demorar 3 horas en cargar approx.\n4. Llevo alrededor de 6 meses utilizandola, y me ha presentado un par de fallas respecto al sonido, he tenido la obligación de reiniciarle, y se ha solucionado.\nBuen producto, para el que busque algo correcto a buen precio.', 'votos_utiles': '4'}, {'calificacion': 5, 'fecha': '02 dic. 2024', 'contenido': 'Excelente producto en relación precio/calidad. Ha cumplido en las tareas en que la he usado como edición de video y toma de apuntes. El lápiz funciona bastante bien.', 'votos_utiles': '3'}]</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>45809.67834961102</v>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_602205-MLA74652847384_022024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_773066-MLA52988770867_122022-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_860664-MLA52988782788_122022-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_944519-MLU73115284216_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_781580-MLU75321470327_032024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_694460-MLU70065260095_062023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_810307-MLU75321420641_032024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_853829-MLU75321391561_032024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_742900-MLU75174250074_032024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_791595-MLU73115624998_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_920640-MLU73115625028_122023-F.webp']</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '07 ago. 2022', 'contenido': 'Feliz con la compra, pedí outemu rojo, que son los clips del teclado. Estos son silenciosos y más suaves que el outemu blue.\nA mí me gusta el teclado silencioso por eso preferí outemu rojo.\nEl teclado tiene retroalimentación de calidad, y se siente la calidad del teclado. Con teclas inborrables porque son de doble inyección.\nMuy feliz con el teclado 100% original. Gracias.', 'votos_utiles': '2'}, {'calificacion': 5, 'fecha': '20 jun. 2022', 'contenido': 'Es un gran teclado, de muy buena construcción y robusto, sin embargo en la publicación dice que vienen con unos switches outemu blue, y vino con unos switches de color rojo de los cuales no se exactamente la referencia. Aun asi me siento conforme con el funcionamiento de este y lo recomiendo.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '06 ene. 2022', 'contenido': 'Buen producto relación calidad precio.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '09 abr. 2024', 'contenido': 'Se ve de muy buena calidad se nota q es de buena construcción espero q dure.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '14 may. 2025', 'contenido': 'Me gustó mucho el producto, bastante sólido se siente de buena construcción y buena calidad, sensación agradable al momento de pulsar las teclas y buena retroiluminación en cada una de las transiciones, recomiendo el producto totalmente.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>45809.68173765656</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LOGITECH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Logitech G413 Se, Teclado Gamer Mecánico Retroiluminado Led Color del teclado Grafito Idioma Inglés</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=1%2BmSDuFEjeCjf5EyjYdV5LjMfAU5owNLHEYv3ks1VKpD0Gs0zZTvdlXGVSqVU2xg%2BncfChY%2BC%2BAAHw37%2F7v%2BEifMiSaJ4p17K3K5XrAXV2HEQv4MYSAql9TGf%2BB9VigDzre5GPNO5v%2F6zUHVGeGXBAb0ww3SZNZsWxcpGcVvIrsd%2FB9RcBs9oHxqv3cI0u2A5f1D5XAcqNDhSB9Ee4tEbShrr0kTBMcGviYSNFBtDMz24KVROBy2GoNoJRTiQzllPVlRY7ZFeIEpVsPwAaYH9fjbFmfU1V5gIZRyKCcxbMScmI71XEgfLilHueoqznPDxM7jHKWZ2mZ8aUMBsW1go4M%2BS3pz44v947MELQdtLTgQZmaOj%2BuRTaK%2FwUJXPB8Ry7l5DOsn%2F5jAlDBrvrDctWkiX2gjoBGot4qHPrJUmglwGID9XabLA%2BDt7KHqJGp0hr8VITlYrO%2FPZwzKfHZwjmqHiPz2iCHepwmXYahnElJoJU8vPqD4mYPua4sSpdiVjfFeAJVVaY6dNadGNXQFdg9EFp5qQ70oXeooPtemL%2BeSjOppfN32ZF%2FYvi1VLZj%2FqkJ1I3UrOHMwwK7IKWHRbWo1C%2FEzAIFqJnqtFRB9MBTDNV2sYdKHQUvdBD7M2P5BRlPeLcQwrh%2BFd3iLqI0e3M4c0COGIs3IIRgUI4IqrBkPWIYO9rePq%2FkwQYpAaIKtMU3poo3JeH%2BbjxHSm3nVpXlKa1rtDmwj2QtiGEhfDa6AX5g%2BzB28X5ZI2r9LSLsbjH1sQdIrBOcQd0uL1Uq97ZWs5JnwPo0oxbkLpeoYVi%2BubPo84aEBdcP0PA225XXI8efe9qSlN4UBfKvI3TgcbAYEua9Xjg8StyPoaG0LTgtFNSSiRFv2fJ7sswbMuBh3imQ2D1nexgmFmkMUgmqsQ12vs2iYADEwmMNaRsnWbesp6x1MIVUPFtuV%2FlBIVhkKCsB2wh39b7M9ZBk%2B3ruWNCHYUzP%2Fjs6rP%2F7GdfF5ZEt3OhCbmUVb&amp;highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO2855290132&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>357135</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_942664-MLA84857255411_052025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_831940-MLA84724971460_052025-F.jpg']</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '06 mar. 2025', 'contenido': 'Es un 10/10.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '26 dic. 2024', 'contenido': 'Excelente teclado, super rápido paea video juegos muy bueno.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '16 sep. 2024', 'contenido': 'Muy buen teclado, excelente para el gaming.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '11 sep. 2024', 'contenido': 'Con respecto al producto era lo que esperaba, con respecto a la transportadora sé que "envia" es económico pero en muchas áreas del territorio nacional es pésima transportadora, se recomienda cambiar.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '07 jun. 2024', 'contenido': 'Es un buen producto suave silencioso buenas y faciles de combinación del teclado para juegos súper rapido.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>45809.68173766883</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Teclado Mecanico Gaming Premium Tkl Rgb - Blue Switches</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolibre.com.co/mclics/clicks/external/MCO/count?a=raxnTiIOfaJGLihafXujD1LfKau1fJt4%2BALVI8%2Bbs57gk4gn%2B0x02l14%2Bit8M7USHQqk8J23Vd7Ela7IruCNXs6Ba7umN1djjbgLKGjPph%2FmF0UKdIhSJWpwIuISvLU34eiNhA2Qz8W8vi%2BClW5rR%2F0zqyi%2BIsWNQ59tjuM%2F8Gy%2F%2F7AcRkW%2BxaQdc52oU37aDBgoxAlqLbTnIYPAkZNeXB2ASeKhGCYMSzORUQFu64NWzbj9X1Ewu69jq6ytRR9tG6BySZ7PqESZlYHXuPWqq3pZy9K740WAlK7N4kMTSHfEht9Pjnm8HkwzsLtvdd1AXZwLRGpirSldH8IrIB29Y6UJlPjl3qcDT%2FHFEV79Rcd7KnS2%2BmNHhRXL9%2F9O03fL4Wur5GvRHtOZPKvRWbWQJLOX595%2FB5tE5CaMf%2BIpmx0rndZOd1aiQMjhEqB0aSnucvngxtVhTqF92xNEu5bSFN5K01hGjQrrYP7qMQ3bmZLdf%2BUzu4wY0qXiYppVcagqcgMKXyyX838k%2FOcuHMCbq7u3O1V%2FbcOqATG8%2FGY909oLtZoV8TvvTOLAV3XjKqNcM%2F1CK83TDb%2FLDBqaYwjB1d3P9dYp0gsnR4jszJnY2jL0ut6oC6Xon8cEjx9jngDpHKfXeKwM%2B6F%2BCFahWXIxzXkcPfV9KIt5nnys%2BEUwxIin993%2FQ4A01WoeagLTABfk2aj2qSMnwP9LIcOvSNEN73fiDov8%2BWR3M%2FCr46AOOfjYcmr2zxiJK7iwJIvoLfyCIzxJWMDPQsihVf6rA2HN6Z6xoDV%2BvzNy7xWBKqOwbxao2uHS%2F8VWRTvzzyA4eZ%2BXuJiTc4eoEDCtpt0VMnnYK0TmNxKNAZr%2FVucsswAhmzh5S%2FYS4gm5wQ3Y33jkQQOIZZUFvSLFK135iqeKhujn19FufKQtndb5FpMSBuhgJ1GVQMMoQb%2FvQ0x9&amp;searchVariation=175176005934&amp;highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>107920</v>
+      </c>
+      <c r="E8" t="n">
+        <v>134900</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>20% OFF</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_713856-MCO83310185804_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_906560-MCO83311522676_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_629139-MCO83311522714_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_952983-MCO83603556415_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_729467-MCO83603556433_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_862622-MCO83311591058_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_649367-MCO83311591070_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_879923-MCO83327889878_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_835523-MCO83311591120_042025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_837709-MCO83603556513_042025-F.webp']</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '21 may. 2025', 'contenido': 'Suena muy lindo y tiene muchos modos de colores, puedes ponerlo solo rojo y varios colores también tiene multicolor a la vez 🥰🥰.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '13 may. 2025', 'contenido': 'Excelente, recomendado 100%.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '31 may. 2025', 'contenido': 'Es un excelente teclado mecánico, tiene una configuración sencilla de las luces de fondo, también trae para personalizar macros en algunas teclas, tiene un sonido aceptable. Es un poco pesado en comparación con otros, muy estético y trae mucha variedad de configuración de luces.\nLo recomiendo mucho si te gustan los teclados mecánicos al 65% para ahorrar espacios.\nDe muy buena calidad.\nVale la penam por el precio.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '29 may. 2025', 'contenido': 'Tremendo, para su valor. Muy bueno. Eso sí, suena un tris duro.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '28 may. 2025', 'contenido': 'Es sorpréndete la calidad que tiene para lo barato que es, la sensación, las luces, el sonido. Es magnifico! 10 de 10.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>45809.68173768006</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Teclado Gamer T-dagger Arena T-tgk321 Qwerty T-dagger Brown Español Color Negro Con Luz Rainbow</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/teclado-gamer-t-dagger-arena-t-tgk321-qwerty-t-dagger-brown-espanol-color-negro-con-luz-rainbow/p/MCO25354558?highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO25354558&amp;position=13&amp;search_layout=stack&amp;type=product&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO1435132381&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>149900</v>
+      </c>
+      <c r="E9" t="n">
+        <v>214143</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>30% OFF</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_829971-MLU72637468711_112023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_846613-MLA79492165647_092024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_815620-MLU74161826881_012024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_916860-MLU72566191648_112023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_980831-MLA79491981591_092024-F.webp']</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '04 feb. 2025', 'contenido': '', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '25 oct. 2024', 'contenido': 'Muy lindo y comodo.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '22 ene. 2025', 'contenido': 'Me parece un exelente producto precio calidad. Los materiales son bueno y el silencioso, me encantó recomendado.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '22 ene. 2025', 'contenido': '', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '25 abr. 2025', 'contenido': 'Un muy buen producto calidad precio, el teclado es bastante silencioso lo cual es perfecto para mí, también es muy cómodo pero tiene dos cositas que no me gustaron.\n1) entiendo el tema de 60% y la combinación de teclas con el fn pero un teclado de este tamaño necesita por obligación un software de configuración de teclas propio prácticamente no se pueden usar las flechas ya que si das fn + w vas a bloquear wasd como flechas de movimiento pero a su misma vez fn + w es flecha arriba si yo solo quiero ir hacia arriba en un texto voy a tener que darle dos veces por lo que va a subir dos veces el cursor en resumen esa combinación me aprece que está mal y no se puede cambiar.\n2) se escucha un poco el rebote de las teclas cuando se usan muy rápido pero esto puede ser tema de los switches a lo mejor con una lubricada se quite pero de fabrica puede ser un poco molesto.\nPero en general es un muy buen teclado cumple exelente su función ya llevo un mes con el usando todos los días y nunca me deja tirado lo recomiendo.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>45809.68173769186</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Teclado Mecánico Gaming Redragon K636clo Rgb Color del teclado Negro Idioma Inglés US</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/teclado-mecanico-gaming-redragon-k636clo-rgb-color-del-teclado-negro-idioma-ingles-us/p/MCO29039269?highlight=true&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO29039269&amp;position=14&amp;search_layout=stack&amp;type=product&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO2772382820&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>210028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_674064-MLU73503205759_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_943483-MLU73411990606_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_651951-MLU73411990618_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_758706-MLU73503205777_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_988320-MLU73502811109_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_891015-MLU73502870103_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_742169-MLU73411931788_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_723670-MLU73503225631_122023-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_629594-MLU77910155149_072024-F.webp']</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '02 mar. 2024', 'contenido': 'Excelente producto, muy bueno, hace falta revisar las macros pero cómo quedo configurado con solo conectarlo estoy feliz. Todas las teclas funcionan a la perfección.', 'votos_utiles': '2'}, {'calificacion': 5, 'fecha': '07 nov. 2024', 'contenido': 'Muy bueno, silencioso, suave y práctico, funcionando perfectamente.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '30 abr. 2024', 'contenido': 'Muy bonito exelente producto lo recomiendo 🔥🔥🔥.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '25 may. 2025', 'contenido': 'Justo lo que estaba buscando, por el precio esta muy bien.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '04 abr. 2025', 'contenido': 'Excelente. Viene con las herramientas para cambiar las teclas. Un producto muy completo y estético, sobre todo por el precio!.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>45809.6817377041</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Teclado Mecánico Gamer Gamepower Suki Tkl Switches necánicos 87 teclas antighosting reposamuñecas magnético</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.mercadolibre.com.co/teclado-mecanico-gamer-gamepower-suki-tkl-switches-necanicos-87-teclas-antighosting-reposamunecas-magnetico/p/MCO45207491?highlight=false&amp;headerTopBrand=false#polycard_client=search-nordic&amp;searchVariation=MCO45207491&amp;position=5&amp;search_layout=stack&amp;type=product&amp;tracking_id=d5bd1a16-2a63-481d-ab07-d7b9f14f3457&amp;wid=MCO1542802747&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>127415</v>
+      </c>
+      <c r="E11" t="n">
+        <v>149900</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>15% OFF</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Envío gratis</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>['https://http2.mlstatic.com/D_NQ_NP_2X_806430-MLA81431205572_122024-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_636597-MLA82479025889_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_752807-MLA82478968071_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_899959-MLA82478941533_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_678323-MLA82478968095_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_762905-MLA82479025859_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_686051-MLA82478941575_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_629643-MLA82478968169_022025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_848904-MLA84026494874_052025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_614756-MLA84321552659_052025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_959549-MLA84321552663_052025-F.webp', 'https://http2.mlstatic.com/D_NQ_NP_2X_739424-MLA84026494876_052025-F.webp']</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>[{'calificacion': 5, 'fecha': '08 abr. 2025', 'contenido': 'Excelente , calidad y todo.', 'votos_utiles': '1'}, {'calificacion': 5, 'fecha': '29 may. 2025', 'contenido': 'Excelente teclado para el precio, el recorrido es bastante alto por lo que no es para todo el mundo y los switches no son tan silenciosos, pero en luces y calidad es excelente, sin contar con que permite extraer keycaps fácilmente y el frente es metálico, muy buen producto.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '10 abr. 2025', 'contenido': '', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '05 may. 2025', 'contenido': 'Muy bueno.', 'votos_utiles': '0'}, {'calificacion': 5, 'fecha': '27 abr. 2025', 'contenido': 'Exelente.', 'votos_utiles': '0'}]</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>45809.68173771294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>